<commit_message>
normalize PANNs: filter unmapped AudioSet labels, enrich GT_KEYWORDS, regen DBs + xlsx
</commit_message>
<xml_diff>
--- a/data/analysis_gemini_2_5_flash_panns/multimodal_event_eval_gemini_2_5_flash_panns_w2_5s_h1_25s.xlsx
+++ b/data/analysis_gemini_2_5_flash_panns/multimodal_event_eval_gemini_2_5_flash_panns_w2_5s_h1_25s.xlsx
@@ -115,10 +115,10 @@
     <t>gunshot_or_explosion(48-240)</t>
   </si>
   <si>
-    <t>sound: speech(0-120), sound: burst_pop(90-150), sound: gunshot_or_explosion(120-180), sound: engine(150-240), visual: enter_or_exit_vehicle(0-0), visual: explosion_visible(120-216), visual: explosion_visible(120-240), visual: gunshot_visible(48-96), visual: physical_altercation(48-96), visual: running(144-168), visual: running(144-168), visual: suspicious_near_vehicle(72-96), visual: suspicious_near_vehicle(96-96), visual: vehicle_collision(216-216), visual: vehicle_collision(216-216), visual: vehicle_collision(216-216)</t>
-  </si>
-  <si>
-    <t>gunshot_or_explosion(60-120)</t>
+    <t>sound: gunshot_or_explosion(90-180), sound: engine(150-240), visual: enter_or_exit_vehicle(0-0), visual: explosion_visible(120-216), visual: explosion_visible(120-240), visual: gunshot_visible(48-96), visual: physical_altercation(48-96), visual: running(144-168), visual: running(144-168), visual: suspicious_near_vehicle(72-96), visual: suspicious_near_vehicle(96-96), visual: vehicle_collision(216-216), visual: vehicle_collision(216-216), visual: vehicle_collision(216-216)</t>
+  </si>
+  <si>
+    <t>gunshot_or_explosion(30-120)</t>
   </si>
   <si>
     <t>gunshot_or_explosion(120-180)</t>
@@ -127,13 +127,13 @@
     <t>gunshot_or_explosion(0-240)</t>
   </si>
   <si>
-    <t>sound: gunshot_or_explosion(0-90), sound: speech(60-150), sound: engine(120-240), visual: explosion_visible(192-240), visual: vehicle_collision(192-240)</t>
+    <t>sound: gunshot_or_explosion(0-90), sound: engine(120-240), visual: explosion_visible(192-240), visual: vehicle_collision(192-240)</t>
   </si>
   <si>
     <t>NO</t>
   </si>
   <si>
-    <t>sound: door(0-90), sound: engine(60-240), visual: enter_or_exit_vehicle(48-96)</t>
+    <t>sound: engine(60-240), visual: enter_or_exit_vehicle(48-96)</t>
   </si>
   <si>
     <t>vehicle_escape(24-168)</t>
@@ -142,19 +142,19 @@
     <t>vehicle_escape(24-96)</t>
   </si>
   <si>
-    <t>sound: horn(0-90), sound: breaking(60-150), sound: engine(120-210), sound: door(180-240)</t>
+    <t>sound: horn(0-90), sound: engine(120-210)</t>
   </si>
   <si>
     <t>vehicle_collision(30-150)</t>
   </si>
   <si>
-    <t>sound: engine(0-60), sound: skidding(30-90), sound: gunshot_or_explosion(60-120), sound: glass_breaking(90-150), sound: speech(120-240)</t>
+    <t>sound: engine(0-60), sound: skidding(30-90), sound: gunshot_or_explosion(60-120), sound: glass_breaking(90-150)</t>
   </si>
   <si>
     <t>vehicle_collision(72-240)</t>
   </si>
   <si>
-    <t>sound: horn(0-60), sound: engine(30-240), sound: gunshot_or_explosion(60-120), sound: breaking(90-150), visual: enter_or_exit_vehicle(120-120), visual: enter_or_exit_vehicle(144-240), visual: suspicious_near_vehicle(144-240), visual: vehicle_collision(72-240), visual: vehicle_collision(72-240)</t>
+    <t>sound: horn(0-60), sound: engine(30-240), sound: gunshot_or_explosion(60-120), visual: enter_or_exit_vehicle(120-120), visual: enter_or_exit_vehicle(144-240), visual: suspicious_near_vehicle(144-240), visual: vehicle_collision(72-240), visual: vehicle_collision(72-240)</t>
   </si>
   <si>
     <t>visual: enter_or_exit_vehicle(48-168), visual: suspicious_near_vehicle(48-192)</t>
@@ -184,7 +184,7 @@
     <t>vehicle_escape(0-240)</t>
   </si>
   <si>
-    <t>sound: skidding(0-90), sound: breaking(60-120), sound: door(90-240)</t>
+    <t>sound: skidding(0-90)</t>
   </si>
   <si>
     <t>visual: enter_or_exit_vehicle(48-168), visual: running(216-240), visual: suspicious_near_vehicle(48-96), visual: suspicious_near_vehicle(168-192)</t>

</xml_diff>